<commit_message>
Add CUSTOMER REVIEWS SURVEY For MILK&PULL.xlsx
</commit_message>
<xml_diff>
--- a/week-1/Ex4A_GTrends.xlsx
+++ b/week-1/Ex4A_GTrends.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\DataAnalytics\week-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D78531D-3551-4B15-A1F0-EFFFF9DEAA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D41E32-CCB3-4629-9C1D-FAD66108BBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="3960" windowWidth="30936" windowHeight="16776" xr2:uid="{D5B6ADBA-CB6F-41C8-B3A4-C3FA1E839BB4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D5B6ADBA-CB6F-41C8-B3A4-C3FA1E839BB4}"/>
   </bookViews>
   <sheets>
     <sheet name="Ex4A_GTrends" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ex4A_GTrends!$A$1:$E$52</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>